<commit_message>
Resolved Failed TestCases - 27Mar2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/06_RewardCatalogue/RewardCatalogue/03_RedemptionSummaryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/06_RewardCatalogue/RewardCatalogue/03_RedemptionSummaryPageTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\06_RewardCatalogue\RewardCatalogue\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15302EED-595F-4E50-A180-5DC6D89A6844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{953F428F-BFBD-44F6-8D63-CA2C626CC1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="137">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -1980,6 +1980,23 @@
   </si>
   <si>
     <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>redemptioncart_clickon_cancelbtn
+catalogue_enter_searchdata
+catalogue_clickon_keyboardsearchicon
+hidekeyboard
+catalogue_enter_qty
+hidekeyboard
+catalogue_clickon_submitbtn
+redemptioncart_clickon_checkoutbtn
+summary_enter_deliveredaddress
+summary_enter_pincode
+summary_enter_district
+summary_enter_panno
+summary_clickon_checkout
+summary_clickon_checkout
+verify_summary_declarationtitle</t>
   </si>
 </sst>
 </file>
@@ -3653,7 +3670,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:18" s="14" customFormat="1" ht="203" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" s="14" customFormat="1" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
         <v>8</v>
       </c>
@@ -3667,7 +3684,7 @@
         <v>30</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="F21" s="11" t="s">
         <v>67</v>

</xml_diff>